<commit_message>
Adiciona 5 vagas de estágio TI/Cyber (pesquisa 16/10/2026)
Novas requisições em acompanhamento, sem duplicar as existentes e
preservando encerradas: XP Inc. (talent pool Segurança da Informação),
Nubank Estágio 2027, CI&T NextGen AI, Tempest (Segurança da Informação)
e Conectas (TI). Dados sincronizados em dados_vagas.json, Estagios.csv e
Estagios.xlsx (hyperlinks, notas de pendências e IDs ocultos preservados);
coluna Inscrito? mantida sem marcações no modelo público.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Estagios.xlsx
+++ b/Estagios.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estágios" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Estágios" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Estágios'!$A$1:$J$50</definedName>
@@ -202,6 +202,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>None</author>
+    <author>None</author>
   </authors>
   <commentList>
     <comment ref="J2" authorId="0" shapeId="0">
@@ -496,6 +497,36 @@
       <text>
         <t>40h semanais obrigatórias no anúncio.
 Prazo: 2026-10-30</t>
+      </text>
+    </comment>
+    <comment ref="J51" authorId="1" shapeId="0">
+      <text>
+        <t>Talent pool de Segurança da Informação — cadastro, não vaga aberta com início definido. Confirmar se aceita estagiário, curso exigido, jornada, bolsa e modelo.
+Prazo: Não informado</t>
+      </text>
+    </comment>
+    <comment ref="J52" authorId="1" shapeId="0">
+      <text>
+        <t>Inscrições de 17 a 30/08/2026 pelo estagio.nubank.com.br; início jan/2027. Exige inglês avançado e prática com ferramentas de IA (ex.: Claude, Cursor, Copilot). Monitorar próximo ciclo.
+Prazo: 30/08/2026 (encerrado)</t>
+      </text>
+    </comment>
+    <comment ref="J53" authorId="1" shapeId="0">
+      <text>
+        <t>Ciclos em 2026 (1º lote com inscrições até 12/01/2026, início mar/2026; ~200 vagas por lote). Remoto/híbrido, 4h ou 6h/dia, formatura 12/2026–07/2027. Confirmar novo ciclo e link oficial no ATS.
+Prazo: 12/01/2026 (1º lote encerrado)</t>
+      </text>
+    </comment>
+    <comment ref="J54" authorId="1" shapeId="0">
+      <text>
+        <t>Programa de estágio em segurança da informação com opção remota e auxílio home office. Ciclo divulgado com inscrições até jan/2025; confirmar abertura atual em estagiotempest.gupy.io.
+Prazo: Não informado</t>
+      </text>
+    </comment>
+    <comment ref="J55" authorId="1" shapeId="0">
+      <text>
+        <t>Edital de mar/2026: bolsa R$1.650, híbrido com 2 dias presenciais, 30h/semana. Confirmar se as inscrições seguem abertas.
+Prazo: Não informado</t>
       </text>
     </comment>
   </commentList>
@@ -791,7 +822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.7109375" customWidth="1" style="1" min="1" max="2"/>
@@ -3465,6 +3496,269 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>Monitorar</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>XP Inc. — Talent Pool Segurança da Informação (2026)</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Abrir vaga</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>Não divulgados</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>São Paulo - SP | A confirmar</t>
+        </is>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>Cyber</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="inlineStr">
+        <is>
+          <t>Banco de talentos</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="inlineStr">
+        <is>
+          <t>V-43B63A264F</t>
+        </is>
+      </c>
+      <c r="L51" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:00:00-03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>Monitorar</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>Nubank — Programa de Estágio 2027 (Tecnologia / Dados / IA)</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Abrir vaga</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>Não divulgados</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>Regiões metro de São Paulo / Campinas / Rio de Janeiro / Belo Horizonte | Híbrido (3 dias escritório / 2 remoto)</t>
+        </is>
+      </c>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>30h/semana</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="J52" s="1" t="inlineStr">
+        <is>
+          <t>Encerrada</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="inlineStr">
+        <is>
+          <t>V-68060AED79</t>
+        </is>
+      </c>
+      <c r="L52" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:00:00-03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>Monitorar</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>CI&amp;T — Programa de Estágio NextGen AI (Desenvolvimento / IA)</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Abrir vaga</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>Não divulgados</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>Brasil | Remoto ou híbrido</t>
+        </is>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>4h ou 6h/dia</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="J53" s="1" t="inlineStr">
+        <is>
+          <t>Confirmar abertura / requisitos</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="inlineStr">
+        <is>
+          <t>V-209B309BAA</t>
+        </is>
+      </c>
+      <c r="L53" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:00:00-03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>Monitorar</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>Tempest Security Intelligence — Estágio em Segurança da Informação</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Abrir vaga</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>Auxílio home office (para atuação remota)</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>Recife - PE / São Paulo - SP | Híbrido; remoto para demais localidades conforme área</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>Cyber</t>
+        </is>
+      </c>
+      <c r="J54" s="1" t="inlineStr">
+        <is>
+          <t>Confirmar abertura / requisitos</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="inlineStr">
+        <is>
+          <t>V-B38185BDA7</t>
+        </is>
+      </c>
+      <c r="L54" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:00:00-03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>Monitorar</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>Conectas Direitos Humanos — Estágio em TI</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Abrir vaga</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>VT; VR; Saúde; Odontológico; Wellhub; Auxílio idiomas; Auxílio home office (híbrido)</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>São Paulo - SP | Híbrido (2 dias presenciais/semana)</t>
+        </is>
+      </c>
+      <c r="H55" s="1" t="inlineStr">
+        <is>
+          <t>30h/semana (6h/dia)</t>
+        </is>
+      </c>
+      <c r="I55" s="1" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="J55" s="1" t="inlineStr">
+        <is>
+          <t>Confirmar abertura / requisitos</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="inlineStr">
+        <is>
+          <t>V-5CAA83691A</t>
+        </is>
+      </c>
+      <c r="L55" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16T12:00:00-03:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J50"/>
   <conditionalFormatting sqref="A2:J50">
@@ -3478,7 +3772,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A50" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Inscrição" prompt="Marque Sim após enviar. Vazio = sem confirmação." type="list">
+    <dataValidation sqref="A2:A55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Inscrição" prompt="Marque Sim após enviar. Vazio = sem confirmação." type="list">
       <formula1>"Sim,Não"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3532,6 +3826,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>

</xml_diff>